<commit_message>
modelos prontos report ajustado
</commit_message>
<xml_diff>
--- a/sensor_potencial_hidrico_ai/model/resultados_modelos_energy.xlsx
+++ b/sensor_potencial_hidrico_ai/model/resultados_modelos_energy.xlsx
@@ -461,38 +461,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'mlp__activation': 'relu', 'mlp__alpha': 0.01, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (10, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 5000, 'mlp__solver': 'lbfgs'}</t>
+          <t>{'mlp__activation': 'relu', 'mlp__alpha': 0.0001, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (15, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 10000, 'mlp__solver': 'lbfgs'}</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0588</v>
+        <v>0.5647</v>
       </c>
       <c r="D2" t="n">
-        <v>32.5282</v>
+        <v>31.0471</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.00      0.00      0.00        99
-           1       0.00      0.00      0.00       104
-           2       0.00      0.00      0.00       112
-           3       0.00      0.00      0.00        86
-           4       0.05      0.42      0.09        88
-           5       0.00      0.00      0.00        98
-           6       0.00      0.00      0.00       101
-           7       0.07      0.06      0.07        94
-           8       0.06      0.58      0.12        99
-           9       0.00      0.00      0.00       105
-          10       0.00      0.00      0.00       121
-          11       0.00      0.00      0.00        99
-          12       0.00      0.00      0.00        94
-          13       0.00      0.00      0.00        97
-          14       0.00      0.00      0.00       102
-          15       0.00      0.00      0.00        91
-          16       0.00      0.00      0.00       110
-    accuracy                           0.06      1700
-   macro avg       0.01      0.06      0.02      1700
-weighted avg       0.01      0.06      0.02      1700
+           0       0.75      0.99      0.86        99
+           1       0.21      0.15      0.18       104
+           2       0.35      0.38      0.36       112
+           3       0.72      0.67      0.70        86
+           4       0.34      0.48      0.40        88
+           5       0.51      0.47      0.49        98
+           6       0.92      0.97      0.95       101
+           7       0.48      0.67      0.56        94
+           8       0.38      0.21      0.27        99
+           9       0.98      1.00      0.99       105
+          10       0.95      0.94      0.95       121
+          11       0.34      0.25      0.29        99
+          12       0.27      0.21      0.24        94
+          13       0.94      1.00      0.97        97
+          14       0.25      0.29      0.27       102
+          15       0.17      0.09      0.12        91
+          16       0.55      0.69      0.62       110
+    accuracy                           0.56      1700
+   macro avg       0.54      0.56      0.54      1700
+weighted avg       0.54      0.56      0.55      1700
 </t>
         </is>
       </c>
@@ -506,38 +506,38 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'scv__C': 10, 'scv__gamma': 0.001, 'scv__kernel': 'rbf', 'scv__random_state': 42}</t>
+          <t>{'scv__C': 10, 'scv__gamma': 0.1, 'scv__kernel': 'rbf', 'scv__random_state': 42}</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1724</v>
+        <v>0.7582</v>
       </c>
       <c r="D3" t="n">
-        <v>44.2294</v>
+        <v>20.2482</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.50      0.13      0.21        99
-           1       0.07      0.01      0.02       104
-           2       0.32      0.06      0.10       112
-           3       0.06      0.87      0.11        86
-           4       0.23      0.03      0.06        88
-           5       0.06      0.01      0.02        98
-           6       0.56      0.22      0.31       101
-           7       0.23      0.05      0.09        94
-           8       0.32      0.06      0.10        99
-           9       0.98      1.00      0.99       105
-          10       0.58      0.06      0.11       121
-          11       0.19      0.03      0.05        99
-          12       0.26      0.05      0.09        94
-          13       0.62      0.22      0.32        97
-          14       0.11      0.02      0.03       102
-          15       0.26      0.08      0.12        91
-          16       0.33      0.09      0.14       110
-    accuracy                           0.17      1700
-   macro avg       0.33      0.18      0.17      1700
-weighted avg       0.34      0.17      0.17      1700
+           0       0.82      0.99      0.90        99
+           1       0.53      0.52      0.52       104
+           2       0.56      0.59      0.58       112
+           3       0.89      0.97      0.93        86
+           4       0.56      0.56      0.56        88
+           5       0.86      0.70      0.78        98
+           6       0.95      0.98      0.97       101
+           7       0.88      0.68      0.77        94
+           8       0.94      0.77      0.84        99
+           9       0.95      1.00      0.97       105
+          10       0.93      0.96      0.94       121
+          11       0.47      0.52      0.49        99
+          12       0.90      0.60      0.72        94
+          13       0.90      1.00      0.95        97
+          14       0.43      0.47      0.45       102
+          15       0.81      0.55      0.65        91
+          16       0.69      0.98      0.81       110
+    accuracy                           0.76      1700
+   macro avg       0.77      0.75      0.75      1700
+weighted avg       0.77      0.76      0.76      1700
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
best parameters finded with roc auc
</commit_message>
<xml_diff>
--- a/sensor_potencial_hidrico_ai/model/resultados_modelos_energy.xlsx
+++ b/sensor_potencial_hidrico_ai/model/resultados_modelos_energy.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,15 +441,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>roc_auc_score</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>mse</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>relatorio_classificacao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>n_combinations</t>
         </is>
@@ -461,43 +466,46 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'mlp__activation': 'relu', 'mlp__alpha': 0.01, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (10, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 5000, 'mlp__solver': 'lbfgs'}</t>
+          <t>{'mlp__activation': 'tanh', 'mlp__alpha': 0.01, 'mlp__early_stopping': True, 'mlp__hidden_layer_sizes': (20, 10), 'mlp__learning_rate': 'constant', 'mlp__learning_rate_init': 0.001, 'mlp__max_iter': 5000, 'mlp__solver': 'adam'}</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0588</v>
+        <v>0.1418</v>
       </c>
       <c r="D2" t="n">
-        <v>32.5282</v>
-      </c>
-      <c r="E2" t="inlineStr">
+        <v>0.637</v>
+      </c>
+      <c r="E2" t="n">
+        <v>51.8347</v>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
-           0       0.00      0.00      0.00        99
-           1       0.00      0.00      0.00       104
+           0       0.12      0.70      0.20        99
+           1       0.12      0.20      0.15       104
            2       0.00      0.00      0.00       112
-           3       0.00      0.00      0.00        86
-           4       0.05      0.42      0.09        88
-           5       0.00      0.00      0.00        98
-           6       0.00      0.00      0.00       101
-           7       0.07      0.06      0.07        94
-           8       0.06      0.58      0.12        99
-           9       0.00      0.00      0.00       105
-          10       0.00      0.00      0.00       121
+           3       0.11      0.02      0.04        86
+           4       0.17      0.01      0.02        88
+           5       0.08      0.08      0.08        98
+           6       0.37      0.07      0.12       101
+           7       0.00      0.00      0.00        94
+           8       0.00      0.00      0.00        99
+           9       0.18      1.00      0.30       105
+          10       0.13      0.02      0.03       121
           11       0.00      0.00      0.00        99
-          12       0.00      0.00      0.00        94
-          13       0.00      0.00      0.00        97
+          12       0.17      0.02      0.04        94
+          13       0.30      0.11      0.16        97
           14       0.00      0.00      0.00       102
-          15       0.00      0.00      0.00        91
+          15       0.10      0.14      0.12        91
           16       0.00      0.00      0.00       110
-    accuracy                           0.06      1700
-   macro avg       0.01      0.06      0.02      1700
-weighted avg       0.01      0.06      0.02      1700
+    accuracy                           0.14      1700
+   macro avg       0.11      0.14      0.07      1700
+weighted avg       0.11      0.14      0.07      1700
 </t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>72</v>
+      <c r="G2" t="n">
+        <v>144</v>
       </c>
     </row>
     <row r="3">
@@ -506,16 +514,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'scv__C': 10, 'scv__gamma': 0.001, 'scv__kernel': 'rbf', 'scv__random_state': 42}</t>
+          <t>{'svc__C': 10, 'svc__gamma': 0.001, 'svc__kernel': 'rbf', 'svc__probability': True, 'svc__random_state': 42}</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>0.1724</v>
       </c>
       <c r="D3" t="n">
+        <v>0.6377</v>
+      </c>
+      <c r="E3" t="n">
         <v>44.2294</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">              precision    recall  f1-score   support
            0       0.50      0.13      0.21        99
@@ -541,7 +552,7 @@
 </t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>